<commit_message>
Update daily indicator data
</commit_message>
<xml_diff>
--- a/930955indicator.xlsx
+++ b/930955indicator.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="8.83203125" customWidth="1" min="1" max="1"/>
@@ -546,7 +546,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20260604</v>
+        <v>20260605</v>
       </c>
       <c r="B2" t="n">
         <v>930955</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>8.68</v>
+        <v>8.74</v>
       </c>
       <c r="H2" t="n">
         <v>10.18</v>
       </c>
       <c r="I2" t="n">
-        <v>5.14</v>
+        <v>5.11</v>
       </c>
       <c r="J2" t="n">
         <v>5.22</v>
@@ -586,7 +586,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20260603</v>
+        <v>20260604</v>
       </c>
       <c r="B3" t="n">
         <v>930955</v>
@@ -612,21 +612,21 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>8.77</v>
+        <v>8.68</v>
       </c>
       <c r="H3" t="n">
-        <v>10.29</v>
+        <v>10.18</v>
       </c>
       <c r="I3" t="n">
-        <v>5.09</v>
+        <v>5.14</v>
       </c>
       <c r="J3" t="n">
-        <v>5.16</v>
+        <v>5.22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20260602</v>
+        <v>20260603</v>
       </c>
       <c r="B4" t="n">
         <v>930955</v>
@@ -652,21 +652,21 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8.83</v>
+        <v>8.77</v>
       </c>
       <c r="H4" t="n">
-        <v>10.38</v>
+        <v>10.29</v>
       </c>
       <c r="I4" t="n">
-        <v>5.05</v>
+        <v>5.09</v>
       </c>
       <c r="J4" t="n">
-        <v>5.12</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20260601</v>
+        <v>20260602</v>
       </c>
       <c r="B5" t="n">
         <v>930955</v>
@@ -695,18 +695,18 @@
         <v>8.83</v>
       </c>
       <c r="H5" t="n">
-        <v>10.43</v>
+        <v>10.38</v>
       </c>
       <c r="I5" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="J5" t="n">
-        <v>5.09</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20260529</v>
+        <v>20260601</v>
       </c>
       <c r="B6" t="n">
         <v>930955</v>
@@ -732,101 +732,101 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>8.73</v>
+        <v>8.83</v>
       </c>
       <c r="H6" t="n">
-        <v>10.26</v>
+        <v>10.43</v>
       </c>
       <c r="I6" t="n">
-        <v>5.11</v>
+        <v>5.06</v>
       </c>
       <c r="J6" t="n">
-        <v>5.18</v>
+        <v>5.09</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>20260529</v>
+      </c>
+      <c r="B7" t="n">
+        <v>930955</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>中证红利低波动100指数</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>红利低波100</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CSI Dividend Low Volatility 100 Index</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Dividend Low Volatility100</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>20260528</v>
       </c>
-      <c r="B7" t="n">
-        <v>930955</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>中证红利低波动100指数</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>红利低波100</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>CSI Dividend Low Volatility 100 Index</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Dividend Low Volatility100</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+      <c r="B8" t="n">
+        <v>930955</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>中证红利低波动100指数</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>红利低波100</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CSI Dividend Low Volatility 100 Index</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dividend Low Volatility100</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H8" t="n">
         <v>10.07</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I8" t="n">
         <v>4.73</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J8" t="n">
         <v>5.33</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>20260527</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>930955</v>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>中证红利低波动100指数</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>红利低波100</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>CSI Dividend Low Volatility 100 Index</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Dividend Low Volatility100</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>8.630000000000001</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>10.16</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>5.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>20260526</v>
+        <v>20260527</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>930955</v>
@@ -852,21 +852,21 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>8.640000000000001</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>10.19</v>
+        <v>10.16</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>4.68</v>
+        <v>4.69</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>5.27</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>20260525</v>
+        <v>20260526</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>930955</v>
@@ -895,7 +895,7 @@
         <v>8.640000000000001</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>10.18</v>
+        <v>10.19</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>4.68</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>20260522</v>
+        <v>20260525</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>930955</v>
@@ -932,21 +932,21 @@
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>8.65</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>10.15</v>
+        <v>10.18</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>4.68</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>5.29</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>20260521</v>
+        <v>20260522</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>930955</v>
@@ -972,21 +972,21 @@
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>8.68</v>
+        <v>8.65</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>10.2</v>
+        <v>10.15</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>4.66</v>
+        <v>4.68</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>5.27</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>20260520</v>
+        <v>20260521</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>930955</v>
@@ -1012,21 +1012,21 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>8.69</v>
+        <v>8.68</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>10.27</v>
+        <v>10.2</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>4.66</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>5.23</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>20260519</v>
+        <v>20260520</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>930955</v>
@@ -1052,21 +1052,21 @@
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>8.789999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>10.34</v>
+        <v>10.27</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4.6</v>
+        <v>4.66</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>5.19</v>
+        <v>5.23</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>20260518</v>
+        <v>20260519</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>930955</v>
@@ -1092,21 +1092,21 @@
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>8.75</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>10.25</v>
+        <v>10.34</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>4.63</v>
+        <v>4.6</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>5.24</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>20260515</v>
+        <v>20260518</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>930955</v>
@@ -1132,21 +1132,21 @@
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>10.31</v>
+        <v>10.25</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>4.6</v>
+        <v>4.63</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>5.21</v>
+        <v>5.24</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>20260514</v>
+        <v>20260515</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>930955</v>
@@ -1172,21 +1172,21 @@
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>8.84</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>10.36</v>
+        <v>10.31</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>4.58</v>
+        <v>4.6</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>5.18</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>20260513</v>
+        <v>20260514</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>930955</v>
@@ -1212,21 +1212,21 @@
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>8.82</v>
+        <v>8.84</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>10.42</v>
+        <v>10.36</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>4.59</v>
+        <v>4.58</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>5.15</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>20260512</v>
+        <v>20260513</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>930955</v>
@@ -1252,13 +1252,13 @@
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>8.890000000000001</v>
+        <v>8.82</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>10.43</v>
+        <v>10.42</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>4.55</v>
+        <v>4.59</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>5.15</v>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>20260511</v>
+        <v>20260512</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>930955</v>
@@ -1292,21 +1292,21 @@
         </is>
       </c>
       <c r="G20" s="3" t="n">
-        <v>8.9</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>10.45</v>
+        <v>10.43</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>4.55</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>5.14</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>20260508</v>
+        <v>20260511</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>930955</v>
@@ -1332,21 +1332,21 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>8.91</v>
+        <v>8.9</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>10.41</v>
+        <v>10.45</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>4.54</v>
+        <v>4.55</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>5.16</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>20260507</v>
+        <v>20260508</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>930955</v>
@@ -1372,21 +1372,21 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>8.9</v>
+        <v>8.91</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>10.4</v>
+        <v>10.41</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>4.55</v>
+        <v>4.54</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>5.17</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>20260506</v>
+        <v>20260507</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>930955</v>
@@ -1412,21 +1412,21 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>8.94</v>
+        <v>8.9</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>10.43</v>
+        <v>10.4</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>4.53</v>
+        <v>4.55</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>5.15</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>20260505</v>
+        <v>20260506</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>930955</v>
@@ -1452,21 +1452,21 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>8.779999999999999</v>
+        <v>8.94</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>9.6</v>
+        <v>10.43</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>4.5</v>
+        <v>4.53</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>5.14</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>20260504</v>
+        <v>20260505</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>930955</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>20260430</v>
+        <v>20260504</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>930955</v>
@@ -1541,6 +1541,46 @@
         <v>4.5</v>
       </c>
       <c r="J26" s="3" t="n">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>20260430</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>930955</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>中证红利低波动100指数</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>红利低波100</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>CSI Dividend Low Volatility 100 Index</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Dividend Low Volatility100</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J27" s="3" t="n">
         <v>5.14</v>
       </c>
     </row>

</xml_diff>